<commit_message>
docs(costing): Resume Builder add-on costing — report + 'Resume Add-on' workbook sheet
5 ATS-safe templates × 3 PDF versions per student per year, costed on the
round-2/3 basis (5,000 students, ₹96/USD, Blaze list prices, Tier-2 Cloud
Run for the headless-Chrome render). Cloud ≈ ₹0.05 per download and under
₹1 per student per year even at full usage; the cost is the ~60 person-day
build. Sheet has three usage scenarios, cap sensitivity, build effort and
add-on pricing at the margin targets; README step 9 added.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/Vriddhi_Costing_Sheet.xlsx
+++ b/docs/Vriddhi_Costing_Sheet.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Pricing &amp; P&amp;L" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Sensitivity" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Build Cost" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Resume Add-on" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;[Red]-&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
@@ -35,6 +36,7 @@
     <numFmt numFmtId="169" formatCode="&quot;₹&quot;#,##0.00;[Red]-&quot;₹&quot;#,##0.00"/>
     <numFmt numFmtId="170" formatCode="0.00&quot; L&quot;"/>
     <numFmt numFmtId="171" formatCode="0.00&quot; Cr&quot;"/>
+    <numFmt numFmtId="172" formatCode="&quot;$&quot;0.0000000"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -121,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,6 +175,13 @@
     <xf numFmtId="165" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -561,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -687,100 +696,112 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>'Resume Add-on' costs the Resume Builder add-on (5 ATS-safe templates × 3 PDF versions per student per year): cloud cost per download, three usage scenarios, build effort, cap sensitivity and the add-on price for a target margin.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Yellow</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Input — edit freely</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Grey</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Formula — recalculates automatically</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Key output</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Blaze plan reminder</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Firestore gives 50,000 reads and 20,000 writes free PER DAY (resets daily, no roll-over), then $0.06 / 100K reads and $0.18 / 100K writes. A 5,000-student college uses ~3.4M reads on a teaching day, so the quota covers ~1.5% — you pay from day one, but the unit prices are tiny.</t>
-        </is>
-      </c>
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>GST</t>
+          <t>Blaze plan reminder</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Cloud prices are ex-GST. Google Cloud India adds 18% GST; set 'GST recoverable' = 1 on Inputs if you claim input credit, else 0 to treat it as a cost. Your invoice to the college carries 18% GST on top of the prices here.</t>
+          <t>Firestore gives 50,000 reads and 20,000 writes free PER DAY (resets daily, no roll-over), then $0.06 / 100K reads and $0.18 / 100K writes. A 5,000-student college uses ~3.4M reads on a teaching day, so the quota covers ~1.5% — you pay from day one, but the unit prices are tiny.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>GST</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>With the default inputs the sheet reproduces docs/COSTING_PLAN_1YEAR_5000_STUDENTS.md: cloud ₹52,266, AI ₹1,16,020, team ₹18,00,000. The only difference is overheads: the report used a flat ₹15,000 'tools' line; the sheet itemises ₹39,660 (Workspace, domain, ₹30,000 travel), so break-even is ₹402 instead of ₹397 per student.</t>
+          <t>Cloud prices are ex-GST. Google Cloud India adds 18% GST; set 'GST recoverable' = 1 on Inputs if you claim input credit, else 0 to treat it as a cost. Your invoice to the college carries 18% GST on top of the prices here.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>Reconciliation</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>With the default inputs the sheet reproduces docs/COSTING_PLAN_1YEAR_5000_STUDENTS.md: cloud ₹52,266, AI ₹1,16,020, team ₹18,00,000. The only difference is overheads: the report used a flat ₹15,000 'tools' line; the sheet itemises ₹39,660 (Workspace, domain, ₹30,000 travel), so break-even is ₹402 instead of ₹397 per student.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>scripts/firebase-yearly-cost-plan.mjs and docs/COSTING_PLAN_1YEAR_5000_STUDENTS.md in the Vriddhi repository. Regenerate this workbook with: python3 scripts/build-costing-sheet.py</t>
         </is>
@@ -1721,6 +1742,1578 @@
       <c r="D36" s="46">
         <f>C36/10000000</f>
         <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F99"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="95" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Resume Builder add-on — 5 ATS-safe templates, 3 PDF versions per template per student per year</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Yellow = edit. A 'download' = one server-rendered PDF version (headless Chrome on Cloud Functions, 2 GiB). Re-downloading an already generated PDF is free and does not consume a credit. Prices: Cloud Run Tier 2 (asia-south1) list prices; Firestore / Storage / Hosting prices come from the Inputs sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>1. Product rules</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>ATS-safe templates offered</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>PDF versions (downloads) allowed per template per student per year</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>per template</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Maximum PDF renders per student per year</t>
+        </is>
+      </c>
+      <c r="C8" s="13">
+        <f>$C$6*$C$7</f>
+        <v/>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>per student</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Add-on price charged to the college per student per year (₹)</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>79</v>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>₹ / student / yr</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>what-if for the P&amp;L rows below; the market-facing anchor is retail resume builders at ₹1,000–2,000 per MONTH per individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>2. Unit costs per PDF render (server-side, enforceable credit)</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Billable seconds per render (Chrome launch + render, incl. cold start share)</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>functions/src/utils/pdfRenderer.ts pattern: launch → setContent → pdf; warm ≈ 3–4 s, cold ≈ 8–10 s</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Function memory</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>GiB</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>the existing api function already runs at 2 GiB for Puppeteer; 512 MiB was OOM-killed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>vCPU per instance</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>vCPU</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Cloud Run Tier 2 vCPU price (request-based billing)</t>
+        </is>
+      </c>
+      <c r="C15" s="47" t="n">
+        <v>3.36e-05</v>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>$ per vCPU-second</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>asia-south1 is a Tier 2 region; Tier 1 (us-central1) is $0.000024</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Cloud Run Tier 2 memory price</t>
+        </is>
+      </c>
+      <c r="C16" s="47" t="n">
+        <v>3.5e-06</v>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>$ per GiB-second</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 is $0.0000025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Requests beyond 2 M free per month</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>$ per million</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Share of render compute absorbed by the Cloud Functions free tier</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="11" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>free tier = 128,571 vCPU-s and 257,142 GiB-s per month in Tier 2; the base app uses ~33K vCPU-s a month, so most months the renders fit entirely. 0 = pay full list price (worst case)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Size of one generated PDF</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>text PDF with 1–2 embedded font subsets; a rasterised (image) PDF would be 5–10× larger AND unreadable by ATS — never ship that</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Average months a generated PDF is kept in Cloud Storage during the year</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>keep every version for 12 months (or until 6 months after graduation); average age over the year ≈ 6 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Free re-downloads of an already generated PDF (per version)</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>per version</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>egress multiplier = 1 + this</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Editing sessions per PDF version</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>sessions</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>students open the editor, tweak, preview — not every session ends in a download</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Firestore writes per editing session (debounced autosave)</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>writes</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>autosave every ~10 s of typing; one resume document per student per template</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Firestore reads per editing session</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>reads</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>resume doc + credit ledger + template meta + profile prefill</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Firestore writes per download (credit transaction + ledger row + audit log)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>writes</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Hosting transfer per session (builder bundle + fonts, cached after the first visit)</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>3. Optional AI assist (bullet rewrite, summary, JD keyword suggestions)</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>AI assist enabled? (1 = yes, 0 = no)</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="11" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Hard cap on AI-assist calls per student per year</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>calls</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>cost guard — same pattern as the study-pack limiter in routes/ai-chat.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Tokens in per call</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Tokens out per call</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Model price — input ($ per 1M tokens)</t>
+        </is>
+      </c>
+      <c r="C33" s="30">
+        <f>'AI Costing'!$B$4</f>
+        <v/>
+      </c>
+      <c r="D33" s="11" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash from the AI Costing sheet; switch to $B$5/$C$5 for flash-lite (≈ 4× cheaper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Model price — output ($ per 1M tokens)</t>
+        </is>
+      </c>
+      <c r="C34" s="30">
+        <f>'AI Costing'!$C$4</f>
+        <v/>
+      </c>
+      <c r="D34" s="11" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>4. Build &amp; run effort (in-house team — already salaried in 'Team &amp; Overheads')</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Loaded cost per person-day (₹)</t>
+        </is>
+      </c>
+      <c r="C37" s="25">
+        <f>30000/22</f>
+        <v/>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>₹ / person-day</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>₹30,000 gross per month ÷ 22 working days. This time is ALREADY paid for in the base plan — it is an allocation, not new cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Agency cost per person-day (₹) — if outsourced instead</t>
+        </is>
+      </c>
+      <c r="C38" s="25">
+        <f>'Build Cost'!$B$6*8</f>
+        <v/>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>₹ / person-day</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>from the Build Cost sheet's hourly rate × 8 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Build contingency</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D39" s="11" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; support per year (template tweaks, credit resets, parser regressions)</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>person-days</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Years over which to spread the build cost</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>5. Build effort — person-days (lean in-house, AI-assisted development)</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="10" t="n"/>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="19" t="inlineStr">
+        <is>
+          <t>Work item</t>
+        </is>
+      </c>
+      <c r="C44" s="19" t="inlineStr">
+        <is>
+          <t>Person-days</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="48" t="inlineStr">
+        <is>
+          <t>Resume data model, per-student documents, security rules, autosave, profile prefill from the student record</t>
+        </is>
+      </c>
+      <c r="C45" s="20" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="48" t="inlineStr">
+        <is>
+          <t>Editor UI — sections (contact, summary, education, internships/experience, projects, skills, certifications, achievements, languages), reorder, live preview, mobile layout</t>
+        </is>
+      </c>
+      <c r="C46" s="20" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="48" t="inlineStr">
+        <is>
+          <t>5 ATS-safe templates — single column, standard headings, real text, A4 + Letter, page-break rules, open-licence fonts (2 days each)</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="48" t="inlineStr">
+        <is>
+          <t>Server-side PDF — dedicated 2 GiB function, credit transaction (render + decrement + ledger in one write), Cloud Storage, signed re-download URLs, watermarked unlimited preview</t>
+        </is>
+      </c>
+      <c r="C48" s="20" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="48" t="inlineStr">
+        <is>
+          <t>ATS checker — rule-based score: sections present, contact block, heading names, no tables/images/columns, length, keyword match against a pasted job description, fix-it hints</t>
+        </is>
+      </c>
+      <c r="C49" s="20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="48" t="inlineStr">
+        <is>
+          <t>AI assist (optional) — bullet rewrite, summary draft, JD keyword suggestions, with the per-student cap and cost guard</t>
+        </is>
+      </c>
+      <c r="C50" s="20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="48" t="inlineStr">
+        <is>
+          <t>Admin &amp; superadmin — enable the add-on per college, template on/off, credits view/reset, usage &amp; download dashboard, per-college export</t>
+        </is>
+      </c>
+      <c r="C51" s="20" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="48" t="inlineStr">
+        <is>
+          <t>QA — run every template through 2–3 open-source resume parsers, device matrix, print fidelity, load test at 20 renders/min</t>
+        </is>
+      </c>
+      <c r="C52" s="20" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Total person-days</t>
+        </is>
+      </c>
+      <c r="C53" s="22">
+        <f>SUM(C45:C52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>With contingency — person-days</t>
+        </is>
+      </c>
+      <c r="C54" s="36">
+        <f>$C$53*(1+$C$39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Person-months (÷ 22) — e.g. one developer for this many months, or two for half</t>
+        </is>
+      </c>
+      <c r="C55" s="36">
+        <f>$C$54/22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Build cost — in-house team time (₹, allocation of salaries already in the plan)</t>
+        </is>
+      </c>
+      <c r="C56" s="26">
+        <f>$C$54*$C$37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Build cost — if given to an agency instead (₹)</t>
+        </is>
+      </c>
+      <c r="C57" s="25">
+        <f>$C$54*$C$38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>6. Yearly cost — three usage scenarios (edit the yellow adoption / usage rows)</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="10" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="10" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>MAX — every student uses all credits</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>EXPECTED</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="F60" s="19" t="inlineStr">
+        <is>
+          <t>How it is computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>Share of students who use the builder at all</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="16" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E61" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>PDF versions per active student per year</t>
+        </is>
+      </c>
+      <c r="C62" s="17">
+        <f>$C$8</f>
+        <v/>
+      </c>
+      <c r="D62" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E62" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>MAX is locked to templates × credits; the other two are your estimate of real behaviour</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>AI-assist calls per active student per year</t>
+        </is>
+      </c>
+      <c r="C63" s="17">
+        <f>$C$30</f>
+        <v/>
+      </c>
+      <c r="D63" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E63" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>MAX = the hard cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>Active students</t>
+        </is>
+      </c>
+      <c r="C64" s="13">
+        <f>Inputs!$C$6*C61</f>
+        <v/>
+      </c>
+      <c r="D64" s="13">
+        <f>Inputs!$C$6*D61</f>
+        <v/>
+      </c>
+      <c r="E64" s="13">
+        <f>Inputs!$C$6*E61</f>
+        <v/>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Inputs!students × adoption</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="32" t="inlineStr">
+        <is>
+          <t>PDF renders per year</t>
+        </is>
+      </c>
+      <c r="C65" s="33">
+        <f>C64*C62</f>
+        <v/>
+      </c>
+      <c r="D65" s="33">
+        <f>D64*D62</f>
+        <v/>
+      </c>
+      <c r="E65" s="33">
+        <f>E64*E62</f>
+        <v/>
+      </c>
+      <c r="F65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>Render compute ($)</t>
+        </is>
+      </c>
+      <c r="C66" s="30">
+        <f>C65*$C$12*($C$14*$C$15+$C$13*$C$16)*(1-$C$18)+C65/1000000*$C$17</f>
+        <v/>
+      </c>
+      <c r="D66" s="30">
+        <f>D65*$C$12*($C$14*$C$15+$C$13*$C$16)*(1-$C$18)+D65/1000000*$C$17</f>
+        <v/>
+      </c>
+      <c r="E66" s="30">
+        <f>E65*$C$12*($C$14*$C$15+$C$13*$C$16)*(1-$C$18)+E65/1000000*$C$17</f>
+        <v/>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>renders × seconds × (vCPU price + GiB × memory price) × (1 − free-tier share) + requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>Cloud Storage — PDFs kept ($)</t>
+        </is>
+      </c>
+      <c r="C67" s="30">
+        <f>C65*$C$19/1024*$C$20*Inputs!$C$30</f>
+        <v/>
+      </c>
+      <c r="D67" s="30">
+        <f>D65*$C$19/1024*$C$20*Inputs!$C$30</f>
+        <v/>
+      </c>
+      <c r="E67" s="30">
+        <f>E65*$C$19/1024*$C$20*Inputs!$C$30</f>
+        <v/>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>renders × MB ÷ 1024 × months stored × $/GB-month</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>Cloud Storage — downloads / re-downloads ($)</t>
+        </is>
+      </c>
+      <c r="C68" s="30">
+        <f>C65*(1+$C$21)*$C$19/1024*Inputs!$C$32</f>
+        <v/>
+      </c>
+      <c r="D68" s="30">
+        <f>D65*(1+$C$21)*$C$19/1024*Inputs!$C$32</f>
+        <v/>
+      </c>
+      <c r="E68" s="30">
+        <f>E65*(1+$C$21)*$C$19/1024*Inputs!$C$32</f>
+        <v/>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>renders × (1 + free re-downloads) × MB ÷ 1024 × $/GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>Firestore reads + writes ($)</t>
+        </is>
+      </c>
+      <c r="C69" s="30">
+        <f>(C65*$C$22*$C$23+C65*$C$25)/100000*Inputs!$C$25+C65*$C$22*$C$24/100000*Inputs!$C$24</f>
+        <v/>
+      </c>
+      <c r="D69" s="30">
+        <f>(D65*$C$22*$C$23+D65*$C$25)/100000*Inputs!$C$25+D65*$C$22*$C$24/100000*Inputs!$C$24</f>
+        <v/>
+      </c>
+      <c r="E69" s="30">
+        <f>(E65*$C$22*$C$23+E65*$C$25)/100000*Inputs!$C$25+E65*$C$22*$C$24/100000*Inputs!$C$24</f>
+        <v/>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>autosave writes + credit writes at $0.18/100K; reads at $0.06/100K (the daily free quota is ignored — conservative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>Hosting transfer — builder bundle &amp; fonts ($)</t>
+        </is>
+      </c>
+      <c r="C70" s="30">
+        <f>C65*$C$22*$C$26/1024*Inputs!$C$34</f>
+        <v/>
+      </c>
+      <c r="D70" s="30">
+        <f>D65*$C$22*$C$26/1024*Inputs!$C$34</f>
+        <v/>
+      </c>
+      <c r="E70" s="30">
+        <f>E65*$C$22*$C$26/1024*Inputs!$C$34</f>
+        <v/>
+      </c>
+      <c r="F70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="32" t="inlineStr">
+        <is>
+          <t>Cloud total ($)</t>
+        </is>
+      </c>
+      <c r="C71" s="49">
+        <f>SUM(C66:C70)</f>
+        <v/>
+      </c>
+      <c r="D71" s="49">
+        <f>SUM(D66:D70)</f>
+        <v/>
+      </c>
+      <c r="E71" s="49">
+        <f>SUM(E66:E70)</f>
+        <v/>
+      </c>
+      <c r="F71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="B72" s="32" t="inlineStr">
+        <is>
+          <t>Cloud total (₹)</t>
+        </is>
+      </c>
+      <c r="C72" s="26">
+        <f>C71*Inputs!$C$23</f>
+        <v/>
+      </c>
+      <c r="D72" s="26">
+        <f>D71*Inputs!$C$23</f>
+        <v/>
+      </c>
+      <c r="E72" s="26">
+        <f>E71*Inputs!$C$23</f>
+        <v/>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>× Inputs!fx. Ex-GST</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>Cloud cost per PDF download (₹)</t>
+        </is>
+      </c>
+      <c r="C73" s="50">
+        <f>IF(C65=0,0,C72/C65)</f>
+        <v/>
+      </c>
+      <c r="D73" s="50">
+        <f>IF(D65=0,0,D72/D65)</f>
+        <v/>
+      </c>
+      <c r="E73" s="50">
+        <f>IF(E65=0,0,E72/E65)</f>
+        <v/>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>the number that answers 'what does one download cost us'</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>Cloud cost per student (₹, all students)</t>
+        </is>
+      </c>
+      <c r="C74" s="29">
+        <f>C72/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="D74" s="29">
+        <f>D72/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="E74" s="29">
+        <f>E72/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>AI assist (₹)</t>
+        </is>
+      </c>
+      <c r="C75" s="25">
+        <f>$C$29*C64*C63*($C$31/1000000*$C$33+$C$32/1000000*$C$34)*Inputs!$C$23</f>
+        <v/>
+      </c>
+      <c r="D75" s="25">
+        <f>$C$29*D64*D63*($C$31/1000000*$C$33+$C$32/1000000*$C$34)*Inputs!$C$23</f>
+        <v/>
+      </c>
+      <c r="E75" s="25">
+        <f>$C$29*E64*E63*($C$31/1000000*$C$33+$C$32/1000000*$C$34)*Inputs!$C$23</f>
+        <v/>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>active × calls × ($ per call) × fx</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; support — team time (₹ per year)</t>
+        </is>
+      </c>
+      <c r="C76" s="25">
+        <f>$C$40*$C$37</f>
+        <v/>
+      </c>
+      <c r="D76" s="25">
+        <f>$C$40*$C$37</f>
+        <v/>
+      </c>
+      <c r="E76" s="25">
+        <f>$C$40*$C$37</f>
+        <v/>
+      </c>
+      <c r="F76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>Build — team time (₹, one-time, year 1)</t>
+        </is>
+      </c>
+      <c r="C77" s="25">
+        <f>$C$56</f>
+        <v/>
+      </c>
+      <c r="D77" s="25">
+        <f>$C$56</f>
+        <v/>
+      </c>
+      <c r="E77" s="25">
+        <f>$C$56</f>
+        <v/>
+      </c>
+      <c r="F77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="B78" s="32" t="inlineStr">
+        <is>
+          <t>YEAR-1 total (cloud + AI + maintenance + full build) (₹)</t>
+        </is>
+      </c>
+      <c r="C78" s="26">
+        <f>C72+C75+C76+C77</f>
+        <v/>
+      </c>
+      <c r="D78" s="26">
+        <f>D72+D75+D76+D77</f>
+        <v/>
+      </c>
+      <c r="E78" s="26">
+        <f>E72+E75+E76+E77</f>
+        <v/>
+      </c>
+      <c r="F78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="32" t="inlineStr">
+        <is>
+          <t>Year-1 cost per student (₹)</t>
+        </is>
+      </c>
+      <c r="C79" s="51">
+        <f>C78/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="D79" s="51">
+        <f>D78/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="E79" s="51">
+        <f>E78/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="B80" s="32" t="inlineStr">
+        <is>
+          <t>Steady-state year (cloud + AI + maintenance, build spread over the amortisation years) (₹)</t>
+        </is>
+      </c>
+      <c r="C80" s="31">
+        <f>C72+C75+C76+C77/$C$41</f>
+        <v/>
+      </c>
+      <c r="D80" s="31">
+        <f>D72+D75+D76+D77/$C$41</f>
+        <v/>
+      </c>
+      <c r="E80" s="31">
+        <f>E72+E75+E76+E77/$C$41</f>
+        <v/>
+      </c>
+      <c r="F80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="B81" s="32" t="inlineStr">
+        <is>
+          <t>Steady-state cost per student (₹)</t>
+        </is>
+      </c>
+      <c r="C81" s="51">
+        <f>C80/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="D81" s="51">
+        <f>D80/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="E81" s="51">
+        <f>E80/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>Of which NEW cash beyond the base plan (cloud + AI only) (₹)</t>
+        </is>
+      </c>
+      <c r="C82" s="25">
+        <f>C72+C75</f>
+        <v/>
+      </c>
+      <c r="D82" s="25">
+        <f>D72+D75</f>
+        <v/>
+      </c>
+      <c r="E82" s="25">
+        <f>E72+E75</f>
+        <v/>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>team time is already in 'Team &amp; Overheads'; this is the only line that changes the Google/AI invoice</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>7. Pricing the add-on (uses margin targets &amp; contingency from Inputs)</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="n"/>
+      <c r="D84" s="10" t="n"/>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="10" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>Price per student for the LOW margin target (year-1 cost basis, + contingency) (₹)</t>
+        </is>
+      </c>
+      <c r="C85" s="50">
+        <f>C79*(1+Inputs!$C$132)/(1-Inputs!$C$129)</f>
+        <v/>
+      </c>
+      <c r="D85" s="50">
+        <f>D79*(1+Inputs!$C$132)/(1-Inputs!$C$129)</f>
+        <v/>
+      </c>
+      <c r="E85" s="50">
+        <f>E79*(1+Inputs!$C$132)/(1-Inputs!$C$129)</f>
+        <v/>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Inputs!m1 / cont</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>Price per student for the HIGH margin target (year-1 cost basis, + contingency) (₹)</t>
+        </is>
+      </c>
+      <c r="C86" s="50">
+        <f>C79*(1+Inputs!$C$132)/(1-Inputs!$C$131)</f>
+        <v/>
+      </c>
+      <c r="D86" s="50">
+        <f>D79*(1+Inputs!$C$132)/(1-Inputs!$C$131)</f>
+        <v/>
+      </c>
+      <c r="E86" s="50">
+        <f>E79*(1+Inputs!$C$132)/(1-Inputs!$C$131)</f>
+        <v/>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Inputs!m3 / cont</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>Revenue at the add-on price above (₹)</t>
+        </is>
+      </c>
+      <c r="C87" s="25">
+        <f>Inputs!$C$6*$C$9</f>
+        <v/>
+      </c>
+      <c r="D87" s="25">
+        <f>Inputs!$C$6*$C$9</f>
+        <v/>
+      </c>
+      <c r="E87" s="25">
+        <f>Inputs!$C$6*$C$9</f>
+        <v/>
+      </c>
+      <c r="F87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="B88" s="32" t="inlineStr">
+        <is>
+          <t>Year-1 gross profit at that price (₹)</t>
+        </is>
+      </c>
+      <c r="C88" s="26">
+        <f>C87-C78</f>
+        <v/>
+      </c>
+      <c r="D88" s="26">
+        <f>D87-D78</f>
+        <v/>
+      </c>
+      <c r="E88" s="26">
+        <f>E87-E78</f>
+        <v/>
+      </c>
+      <c r="F88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="B89" s="32" t="inlineStr">
+        <is>
+          <t>Year-1 gross margin at that price</t>
+        </is>
+      </c>
+      <c r="C89" s="44">
+        <f>IF(C87=0,0,C88/C87)</f>
+        <v/>
+      </c>
+      <c r="D89" s="44">
+        <f>IF(D87=0,0,D88/D87)</f>
+        <v/>
+      </c>
+      <c r="E89" s="44">
+        <f>IF(E87=0,0,E88/E87)</f>
+        <v/>
+      </c>
+      <c r="F89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>If bundled free into the base price: gross-margin points it costs on the base price</t>
+        </is>
+      </c>
+      <c r="C90" s="35">
+        <f>C79/'Pricing &amp; P&amp;L'!$B$4</f>
+        <v/>
+      </c>
+      <c r="D90" s="35">
+        <f>D79/'Pricing &amp; P&amp;L'!$B$4</f>
+        <v/>
+      </c>
+      <c r="E90" s="35">
+        <f>E79/'Pricing &amp; P&amp;L'!$B$4</f>
+        <v/>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>year-1 cost per student ÷ the price on 'Pricing &amp; P&amp;L'</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>8. What the cap actually changes — cloud cost per year if every EXPECTED-adoption student used every credit</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="n"/>
+      <c r="D92" s="10" t="n"/>
+      <c r="E92" s="10" t="n"/>
+      <c r="F92" s="10" t="n"/>
+    </row>
+    <row r="93">
+      <c r="B93" s="19" t="inlineStr">
+        <is>
+          <t>Credits per template</t>
+        </is>
+      </c>
+      <c r="C93" s="19" t="inlineStr">
+        <is>
+          <t>Renders per year</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>Cloud cost per year (₹)</t>
+        </is>
+      </c>
+      <c r="E93" s="19" t="inlineStr">
+        <is>
+          <t>Cloud cost per student (₹)</t>
+        </is>
+      </c>
+      <c r="F93" s="19" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C94" s="13">
+        <f>Inputs!$C$6*$D$61*$C$6*B94</f>
+        <v/>
+      </c>
+      <c r="D94" s="27">
+        <f>C94*$D$73</f>
+        <v/>
+      </c>
+      <c r="E94" s="29">
+        <f>D94/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>one final version per template</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C95" s="13">
+        <f>Inputs!$C$6*$D$61*$C$6*B95</f>
+        <v/>
+      </c>
+      <c r="D95" s="27">
+        <f>C95*$D$73</f>
+        <v/>
+      </c>
+      <c r="E95" s="29">
+        <f>D95/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="B96" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C96" s="13">
+        <f>Inputs!$C$6*$D$61*$C$6*B96</f>
+        <v/>
+      </c>
+      <c r="D96" s="27">
+        <f>C96*$D$73</f>
+        <v/>
+      </c>
+      <c r="E96" s="29">
+        <f>D96/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>the proposed rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C97" s="13">
+        <f>Inputs!$C$6*$D$61*$C$6*B97</f>
+        <v/>
+      </c>
+      <c r="D97" s="27">
+        <f>C97*$D$73</f>
+        <v/>
+      </c>
+      <c r="E97" s="29">
+        <f>D97/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="B98" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C98" s="13">
+        <f>Inputs!$C$6*$D$61*$C$6*B98</f>
+        <v/>
+      </c>
+      <c r="D98" s="27">
+        <f>C98*$D$73</f>
+        <v/>
+      </c>
+      <c r="E98" s="29">
+        <f>D98/Inputs!$C$6</f>
+        <v/>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>≈ unlimited in practice</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>The cap is a product and pricing lever (scarcity, top-up revenue, abuse control) — not a cost lever. Even ten credits per template cost a few thousand rupees a year across 5,000 students.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>